<commit_message>
Actualizar datos STPS a marzo 2026 e incorporar datos SCIAN feb-mar
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excels/negociaciones_central.xlsx
+++ b/excels/negociaciones_central.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conasamigobmx-my.sharepoint.com/personal/hector_soto_conasami_gob_mx/Documents/Escritorio/Negociación laboral/excels/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conasamigobmx-my.sharepoint.com/personal/hector_soto_conasami_gob_mx/Documents/Escritorio/CAEL/Informes/Negociación laboral/excels/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{5609D626-6F2A-4FE2-BE94-FAEDC07AE0CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E0E33AE-F00C-425D-887C-29717185F1B9}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{52EB8C62-1894-4404-AE2B-DF84851872F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7799443C-7AC9-481E-BF68-D62CFDAE644A}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ctm" sheetId="3" r:id="rId1"/>
@@ -515,7 +515,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G458"/>
+  <dimension ref="A1:G460"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.265625" bestFit="1" customWidth="1"/>
@@ -11046,17 +11046,63 @@
       <c r="C458" s="2">
         <v>2026</v>
       </c>
-      <c r="D458" s="2">
-        <v>5.1138185918900003</v>
+      <c r="D458" s="3">
+        <v>5.1011995238169998</v>
       </c>
       <c r="E458">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F458">
-        <v>59413</v>
-      </c>
-      <c r="G458" s="2">
-        <v>9.0990000504940003</v>
+        <v>61321</v>
+      </c>
+      <c r="G458" s="3">
+        <v>9.0859025456199998</v>
+      </c>
+    </row>
+    <row r="459" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A459" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B459" s="2">
+        <v>2</v>
+      </c>
+      <c r="C459" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D459" s="3">
+        <v>2.1471533185239999</v>
+      </c>
+      <c r="E459">
+        <v>156</v>
+      </c>
+      <c r="F459">
+        <v>97242</v>
+      </c>
+      <c r="G459" s="3">
+        <v>6.2565723658500003</v>
+      </c>
+    </row>
+    <row r="460" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A460" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B460" s="2">
+        <v>3</v>
+      </c>
+      <c r="C460" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D460" s="3">
+        <v>2.0282997961799998</v>
+      </c>
+      <c r="E460">
+        <v>115</v>
+      </c>
+      <c r="F460">
+        <v>60838</v>
+      </c>
+      <c r="G460" s="3">
+        <v>6.7081069397409996</v>
       </c>
     </row>
   </sheetData>
@@ -11743,16 +11789,16 @@
         <v>2026</v>
       </c>
       <c r="B40" s="2">
-        <v>2.1894025841550002</v>
+        <v>2.7195310456340001</v>
       </c>
       <c r="C40" s="2">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="D40" s="2">
-        <v>2941</v>
+        <v>27830</v>
       </c>
       <c r="E40" s="2">
-        <v>6.063709622577</v>
+        <v>7.0492748832189998</v>
       </c>
     </row>
   </sheetData>
@@ -11762,7 +11808,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:G458"/>
+  <dimension ref="A1:G460"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.73046875" bestFit="1" customWidth="1"/>
@@ -22293,17 +22339,63 @@
       <c r="C458" s="2">
         <v>2026</v>
       </c>
-      <c r="D458" s="2">
-        <v>2.9012078998969999</v>
+      <c r="D458" s="3">
+        <v>2.8700612368849998</v>
       </c>
       <c r="E458">
         <v>60</v>
       </c>
       <c r="F458">
-        <v>53545</v>
-      </c>
-      <c r="G458" s="2">
-        <v>6.8025027546920001</v>
+        <v>54330</v>
+      </c>
+      <c r="G458" s="3">
+        <v>6.7701752254730003</v>
+      </c>
+    </row>
+    <row r="459" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A459" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B459" s="2">
+        <v>2</v>
+      </c>
+      <c r="C459" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D459" s="3">
+        <v>3.375555016316</v>
+      </c>
+      <c r="E459">
+        <v>81</v>
+      </c>
+      <c r="F459">
+        <v>59755</v>
+      </c>
+      <c r="G459" s="3">
+        <v>7.5343931051790003</v>
+      </c>
+    </row>
+    <row r="460" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A460" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B460" s="2">
+        <v>3</v>
+      </c>
+      <c r="C460" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D460" s="3">
+        <v>2.3423152355810002</v>
+      </c>
+      <c r="E460">
+        <v>60</v>
+      </c>
+      <c r="F460">
+        <v>89035</v>
+      </c>
+      <c r="G460" s="3">
+        <v>7.0365255236699999</v>
       </c>
     </row>
   </sheetData>
@@ -22990,16 +23082,16 @@
         <v>2026</v>
       </c>
       <c r="B40" s="2">
-        <v>2.9012078998969999</v>
+        <v>2.7874397105150002</v>
       </c>
       <c r="C40" s="2">
-        <v>60</v>
+        <v>201</v>
       </c>
       <c r="D40" s="2">
-        <v>53545</v>
+        <v>203120</v>
       </c>
       <c r="E40" s="2">
-        <v>6.8025027546920001</v>
+        <v>7.1117483753439998</v>
       </c>
     </row>
   </sheetData>
@@ -23009,7 +23101,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:G457"/>
+  <dimension ref="A1:G460"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.73046875" bestFit="1" customWidth="1"/>
@@ -33528,6 +33620,75 @@
       </c>
       <c r="G457">
         <v>6.38</v>
+      </c>
+    </row>
+    <row r="458" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A458" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B458" s="2">
+        <v>1</v>
+      </c>
+      <c r="C458" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D458" s="2">
+        <v>0</v>
+      </c>
+      <c r="E458" s="2">
+        <v>0</v>
+      </c>
+      <c r="F458" s="2">
+        <v>0</v>
+      </c>
+      <c r="G458" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="459" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A459" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B459" s="2">
+        <v>2</v>
+      </c>
+      <c r="C459" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D459" s="2">
+        <v>0</v>
+      </c>
+      <c r="E459" s="2">
+        <v>0</v>
+      </c>
+      <c r="F459" s="2">
+        <v>0</v>
+      </c>
+      <c r="G459" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="460" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A460" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B460" s="2">
+        <v>3</v>
+      </c>
+      <c r="C460" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D460" s="2">
+        <v>0.98791301757500005</v>
+      </c>
+      <c r="E460" s="2">
+        <v>1</v>
+      </c>
+      <c r="F460" s="2">
+        <v>3357</v>
+      </c>
+      <c r="G460" s="2">
+        <v>5.62</v>
       </c>
     </row>
   </sheetData>
@@ -34214,16 +34375,16 @@
         <v>2026</v>
       </c>
       <c r="B40" s="2">
-        <v>0</v>
+        <v>0.98791301757500005</v>
       </c>
       <c r="C40" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D40" s="2">
-        <v>0</v>
+        <v>3357</v>
       </c>
       <c r="E40" s="2">
-        <v>0</v>
+        <v>5.62</v>
       </c>
     </row>
   </sheetData>
@@ -34910,16 +35071,16 @@
         <v>2026</v>
       </c>
       <c r="B40" s="2">
-        <v>5.1138185918900003</v>
+        <v>2.9398309123469999</v>
       </c>
       <c r="C40" s="2">
-        <v>119</v>
+        <v>392</v>
       </c>
       <c r="D40" s="2">
-        <v>59413</v>
+        <v>219401</v>
       </c>
       <c r="E40" s="2">
-        <v>9.0990000504940003</v>
+        <v>7.1725564149660004</v>
       </c>
     </row>
   </sheetData>
@@ -34929,7 +35090,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:G458"/>
+  <dimension ref="A1:G460"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.73046875" bestFit="1" customWidth="1"/>
@@ -45460,17 +45621,63 @@
       <c r="C458" s="2">
         <v>2026</v>
       </c>
-      <c r="D458" s="2">
-        <v>5.2215082676550004</v>
+      <c r="D458" s="3">
+        <v>5.3663832001199996</v>
       </c>
       <c r="E458">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F458">
-        <v>6471</v>
-      </c>
-      <c r="G458" s="2">
-        <v>9.2107726781019998</v>
+        <v>6631</v>
+      </c>
+      <c r="G458" s="3">
+        <v>9.3611400995319993</v>
+      </c>
+    </row>
+    <row r="459" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A459" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B459" s="2">
+        <v>2</v>
+      </c>
+      <c r="C459" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D459" s="3">
+        <v>2.5908531268539998</v>
+      </c>
+      <c r="E459">
+        <v>52</v>
+      </c>
+      <c r="F459">
+        <v>18533</v>
+      </c>
+      <c r="G459" s="3">
+        <v>6.7181222683859998</v>
+      </c>
+    </row>
+    <row r="460" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A460" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B460" s="2">
+        <v>3</v>
+      </c>
+      <c r="C460" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D460" s="3">
+        <v>8.0132271141379992</v>
+      </c>
+      <c r="E460">
+        <v>20</v>
+      </c>
+      <c r="F460">
+        <v>6019</v>
+      </c>
+      <c r="G460" s="3">
+        <v>12.967549426814999</v>
       </c>
     </row>
   </sheetData>
@@ -46157,16 +46364,16 @@
         <v>2026</v>
       </c>
       <c r="B40" s="2">
-        <v>5.2215082676550004</v>
+        <v>4.2277004136859997</v>
       </c>
       <c r="C40" s="2">
-        <v>21</v>
+        <v>96</v>
       </c>
       <c r="D40" s="2">
-        <v>6471</v>
+        <v>31183</v>
       </c>
       <c r="E40" s="2">
-        <v>9.2107726781019998</v>
+        <v>8.4864304268349997</v>
       </c>
     </row>
   </sheetData>
@@ -46176,7 +46383,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G458"/>
+  <dimension ref="A1:G460"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.73046875" bestFit="1" customWidth="1"/>
@@ -56707,17 +56914,63 @@
       <c r="C458" s="2">
         <v>2026</v>
       </c>
-      <c r="D458" s="2">
-        <v>5.2697538014919996</v>
+      <c r="D458" s="3">
+        <v>4.5949170671420001</v>
       </c>
       <c r="E458">
+        <v>10</v>
+      </c>
+      <c r="F458">
+        <v>7283</v>
+      </c>
+      <c r="G458" s="3">
+        <v>8.560425648771</v>
+      </c>
+    </row>
+    <row r="459" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A459" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B459" s="2">
+        <v>2</v>
+      </c>
+      <c r="C459" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D459" s="3">
+        <v>2.5669725705320001</v>
+      </c>
+      <c r="E459">
+        <v>18</v>
+      </c>
+      <c r="F459">
+        <v>3828</v>
+      </c>
+      <c r="G459" s="3">
+        <v>6.6932810867289998</v>
+      </c>
+    </row>
+    <row r="460" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A460" s="1">
+        <v>46447</v>
+      </c>
+      <c r="B460" s="2">
+        <v>3</v>
+      </c>
+      <c r="C460" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D460" s="3">
+        <v>4.5746138953940001</v>
+      </c>
+      <c r="E460">
         <v>9</v>
       </c>
-      <c r="F458">
-        <v>7234</v>
-      </c>
-      <c r="G458" s="2">
-        <v>9.2608473873369999</v>
+      <c r="F460">
+        <v>6405</v>
+      </c>
+      <c r="G460" s="3">
+        <v>9.3712146760340005</v>
       </c>
     </row>
   </sheetData>
@@ -57404,16 +57657,16 @@
         <v>2026</v>
       </c>
       <c r="B40" s="2">
-        <v>5.2697538014919996</v>
+        <v>4.1442997259640002</v>
       </c>
       <c r="C40" s="2">
-        <v>9</v>
+        <v>37</v>
       </c>
       <c r="D40" s="2">
-        <v>7234</v>
+        <v>17516</v>
       </c>
       <c r="E40" s="2">
-        <v>9.2608473873369999</v>
+        <v>8.4488519068280006</v>
       </c>
     </row>
   </sheetData>
@@ -57423,7 +57676,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G458"/>
+  <dimension ref="A1:G460"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.73046875" bestFit="1" customWidth="1"/>
@@ -67954,7 +68207,7 @@
       <c r="C458" s="2">
         <v>2026</v>
       </c>
-      <c r="D458" s="2">
+      <c r="D458" s="3">
         <v>2.109125404597</v>
       </c>
       <c r="E458">
@@ -67963,8 +68216,54 @@
       <c r="F458">
         <v>12049</v>
       </c>
-      <c r="G458">
-        <v>7.5</v>
+      <c r="G458" s="3">
+        <v>5.9803900738650002</v>
+      </c>
+    </row>
+    <row r="459" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A459" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B459" s="2">
+        <v>2</v>
+      </c>
+      <c r="C459" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D459" s="3">
+        <v>3.4224655262689998</v>
+      </c>
+      <c r="E459">
+        <v>4</v>
+      </c>
+      <c r="F459">
+        <v>17187</v>
+      </c>
+      <c r="G459" s="3">
+        <v>7.5831907837310002</v>
+      </c>
+    </row>
+    <row r="460" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A460" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B460" s="2">
+        <v>3</v>
+      </c>
+      <c r="C460" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D460" s="3">
+        <v>2.0376445961990002</v>
+      </c>
+      <c r="E460">
+        <v>4</v>
+      </c>
+      <c r="F460">
+        <v>3368</v>
+      </c>
+      <c r="G460" s="3">
+        <v>6.717880047505</v>
       </c>
     </row>
   </sheetData>
@@ -68651,16 +68950,16 @@
         <v>2026</v>
       </c>
       <c r="B40" s="2">
-        <v>5.9803900738650002</v>
+        <v>2.7940606674019999</v>
       </c>
       <c r="C40" s="2">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="D40" s="2">
-        <v>12049</v>
+        <v>32604</v>
       </c>
       <c r="E40" s="2">
-        <v>2.109125404597</v>
+        <v>6.9014795730580003</v>
       </c>
     </row>
   </sheetData>
@@ -68670,7 +68969,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="A1:G458"/>
+  <dimension ref="A1:G460"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.73046875" bestFit="1" customWidth="1"/>
@@ -79201,17 +79500,63 @@
       <c r="C458" s="2">
         <v>2026</v>
       </c>
-      <c r="D458" s="2">
-        <v>2.1894025841550002</v>
+      <c r="D458" s="3">
+        <v>2.3514759078209999</v>
       </c>
       <c r="E458">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F458">
-        <v>2941</v>
-      </c>
-      <c r="G458" s="2">
-        <v>6.063709622577</v>
+        <v>2864</v>
+      </c>
+      <c r="G458" s="3">
+        <v>6.2319273743009997</v>
+      </c>
+    </row>
+    <row r="459" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A459" s="1">
+        <v>46054</v>
+      </c>
+      <c r="B459" s="2">
+        <v>2</v>
+      </c>
+      <c r="C459" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D459" s="3">
+        <v>2.719492004748</v>
+      </c>
+      <c r="E459">
+        <v>48</v>
+      </c>
+      <c r="F459">
+        <v>14321</v>
+      </c>
+      <c r="G459" s="3">
+        <v>6.8519363172960004</v>
+      </c>
+    </row>
+    <row r="460" spans="1:7" x14ac:dyDescent="0.45">
+      <c r="A460" s="1">
+        <v>46082</v>
+      </c>
+      <c r="B460" s="2">
+        <v>3</v>
+      </c>
+      <c r="C460" s="2">
+        <v>2026</v>
+      </c>
+      <c r="D460" s="3">
+        <v>2.8186075152650001</v>
+      </c>
+      <c r="E460">
+        <v>27</v>
+      </c>
+      <c r="F460">
+        <v>10645</v>
+      </c>
+      <c r="G460" s="3">
+        <v>7.5346641615780001</v>
       </c>
     </row>
   </sheetData>
@@ -79220,6 +79565,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101008FF9D60EAC15C74AB5D052FF9D77E5BD" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="f95571b9953812dd2fdc4cb3d4990df1">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="131f92be-fc8f-4520-9a64-c4bcb115a629" xmlns:ns4="567dafe5-a41b-4f34-91e8-c3ec40d430cf" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ccd401f49274f34ab9c1e94fafb5be50" ns3:_="" ns4:_="">
     <xsd:import namespace="131f92be-fc8f-4520-9a64-c4bcb115a629"/>
@@ -79460,7 +79814,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_activity xmlns="131f92be-fc8f-4520-9a64-c4bcb115a629" xsi:nil="true"/>
@@ -79468,16 +79822,15 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800F2731-B0A5-464D-91BF-8869F509D4CB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{187BCF11-EB27-42FC-89CB-8D91C498B3CE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -79496,7 +79849,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B62C67E2-B4FF-40AE-8CC2-DF27384F2193}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
@@ -79511,12 +79864,4 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800F2731-B0A5-464D-91BF-8869F509D4CB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Cambio de altura a graficas y corrección de un excel.
</commit_message>
<xml_diff>
--- a/excels/negociaciones_central.xlsx
+++ b/excels/negociaciones_central.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://conasamigobmx-my.sharepoint.com/personal/hector_soto_conasami_gob_mx/Documents/Escritorio/CAEL/Informes/Negociación laboral/excels/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{52EB8C62-1894-4404-AE2B-DF84851872F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7799443C-7AC9-481E-BF68-D62CFDAE644A}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="13_ncr:1_{52EB8C62-1894-4404-AE2B-DF84851872F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5B0F3A28-53F7-4D85-B603-0D781E3D2D5F}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ctm" sheetId="3" r:id="rId1"/>
@@ -56952,7 +56952,7 @@
     </row>
     <row r="460" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A460" s="1">
-        <v>46447</v>
+        <v>46082</v>
       </c>
       <c r="B460" s="2">
         <v>3</v>
@@ -79565,12 +79565,11 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="131f92be-fc8f-4520-9a64-c4bcb115a629" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -79815,17 +79814,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="131f92be-fc8f-4520-9a64-c4bcb115a629" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800F2731-B0A5-464D-91BF-8869F509D4CB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B62C67E2-B4FF-40AE-8CC2-DF27384F2193}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="131f92be-fc8f-4520-9a64-c4bcb115a629"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="567dafe5-a41b-4f34-91e8-c3ec40d430cf"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -79850,18 +79859,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B62C67E2-B4FF-40AE-8CC2-DF27384F2193}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{800F2731-B0A5-464D-91BF-8869F509D4CB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="131f92be-fc8f-4520-9a64-c4bcb115a629"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="567dafe5-a41b-4f34-91e8-c3ec40d430cf"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>